<commit_message>
cleanup planning view sheets, remove unnecessary ActiveX textbox
</commit_message>
<xml_diff>
--- a/Template_Without_VBA/TemplateWithoutVBA.xlsx
+++ b/Template_Without_VBA/TemplateWithoutVBA.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\I519576\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\I334271\OneDrive - SAP SE\Shares\New templates to share\Work files without VBA template\Upload\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37241434-039C-4692-AA01-DF631EA1AD02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A776317C-85BD-4809-A56C-C15B2DFBD53B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="374" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -566,14 +566,12 @@
       <color rgb="FF000000"/>
       <name val="Segoe UI"/>
       <family val="2"/>
-      <charset val="238"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="238"/>
     </font>
   </fonts>
   <fills count="8">
@@ -1149,32 +1147,7 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
@@ -1185,10 +1158,6 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1205,12 +1174,28 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1221,12 +1206,25 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="5"/>
@@ -1279,18 +1277,6 @@
 
 <file path=xl/activeX/activeX3.xml><?xml version="1.0" encoding="utf-8"?>
 <ax:ocx xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ax:classid="{8BD21D40-EC42-11CE-9E0D-00AA006002F3}" ax:persistence="persistStreamInit" r:id="rId1"/>
-</file>
-
-<file path=xl/activeX/activeX4.xml><?xml version="1.0" encoding="utf-8"?>
-<ax:ocx xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ax:classid="{8BD21D10-EC42-11CE-9E0D-00AA006002F3}" ax:persistence="persistStreamInit" r:id="rId1"/>
-</file>
-
-<file path=xl/activeX/activeX5.xml><?xml version="1.0" encoding="utf-8"?>
-<ax:ocx xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ax:classid="{8BD21D10-EC42-11CE-9E0D-00AA006002F3}" ax:persistence="persistStreamInit" r:id="rId1"/>
-</file>
-
-<file path=xl/activeX/activeX6.xml><?xml version="1.0" encoding="utf-8"?>
-<ax:ocx xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ax:classid="{8BD21D10-EC42-11CE-9E0D-00AA006002F3}" ax:persistence="persistStreamInit" r:id="rId1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1605,7 +1591,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -1691,7 +1677,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -1777,7 +1763,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -1863,7 +1849,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -1949,7 +1935,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -2092,7 +2078,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -2178,7 +2164,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -2264,7 +2250,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -2350,7 +2336,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -2436,7 +2422,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -2522,7 +2508,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -2608,7 +2594,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -2694,7 +2680,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -2763,7 +2749,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -2850,7 +2836,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -2936,7 +2922,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -3022,7 +3008,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -3108,7 +3094,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -3194,7 +3180,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -3263,7 +3249,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -3407,7 +3393,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -3493,7 +3479,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -3579,7 +3565,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -3665,7 +3651,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -3751,7 +3737,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -3837,7 +3823,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -3923,7 +3909,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -3992,7 +3978,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -4062,7 +4048,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -4132,7 +4118,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -4202,7 +4188,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -4272,7 +4258,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -4342,7 +4328,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -4412,7 +4398,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -4482,7 +4468,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -4552,7 +4538,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -4622,7 +4608,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -4692,7 +4678,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -4762,7 +4748,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -4832,7 +4818,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -4902,7 +4888,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -4972,7 +4958,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -5042,7 +5028,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -5129,7 +5115,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -5215,7 +5201,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -5301,7 +5287,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-GB" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -5367,68 +5353,6 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor>
-        <xdr:from>
-          <xdr:col>0</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>0</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>0</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>0</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="3093" name="FPMExcelClientSheetOptionstb1" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s3093"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-0000150C0000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:solidFill>
-              <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:solidFill>
-                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
-                  </a:solidFill>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
 </xdr:wsDr>
 </file>
 
@@ -5478,126 +5402,6 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor>
-        <xdr:from>
-          <xdr:col>0</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>0</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>0</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>0</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="5121" name="FPMExcelClientSheetOptionstb1" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s5121"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000001140000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:solidFill>
-              <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:solidFill>
-                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
-                  </a:solidFill>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="absolute">
-        <xdr:from>
-          <xdr:col>8</xdr:col>
-          <xdr:colOff>76200</xdr:colOff>
-          <xdr:row>5</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>8</xdr:col>
-          <xdr:colOff>85725</xdr:colOff>
-          <xdr:row>5</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="5127" name="TextBox2" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s5127"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000007140000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:noFill/>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
 </xdr:wsDr>
 </file>
 
@@ -5913,19 +5717,19 @@
   <sheetData>
     <row r="1" spans="1:17" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2"/>
-      <c r="B1" s="52" t="s">
+      <c r="B1" s="71" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
-      <c r="F1" s="52"/>
-      <c r="G1" s="52"/>
-      <c r="H1" s="52"/>
-      <c r="I1" s="52"/>
-      <c r="J1" s="52"/>
-      <c r="K1" s="52"/>
-      <c r="L1" s="52"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="71"/>
+      <c r="K1" s="71"/>
+      <c r="L1" s="71"/>
     </row>
     <row r="2" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="28" t="s">
@@ -5975,43 +5779,43 @@
     </row>
     <row r="5" spans="1:17" ht="28.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
-      <c r="B5" s="53" t="s">
+      <c r="B5" s="64" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="54"/>
-      <c r="D5" s="54"/>
-      <c r="E5" s="54"/>
-      <c r="F5" s="54"/>
-      <c r="G5" s="54"/>
-      <c r="H5" s="54"/>
-      <c r="I5" s="54"/>
-      <c r="J5" s="54"/>
-      <c r="K5" s="54"/>
-      <c r="L5" s="55"/>
+      <c r="C5" s="65"/>
+      <c r="D5" s="65"/>
+      <c r="E5" s="65"/>
+      <c r="F5" s="65"/>
+      <c r="G5" s="65"/>
+      <c r="H5" s="65"/>
+      <c r="I5" s="65"/>
+      <c r="J5" s="65"/>
+      <c r="K5" s="65"/>
+      <c r="L5" s="66"/>
       <c r="Q5" s="19" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="28.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
-      <c r="B6" s="56"/>
-      <c r="C6" s="57"/>
-      <c r="D6" s="57"/>
-      <c r="E6" s="57"/>
-      <c r="F6" s="57"/>
-      <c r="G6" s="57"/>
-      <c r="H6" s="57"/>
-      <c r="I6" s="57"/>
-      <c r="J6" s="57"/>
-      <c r="K6" s="57"/>
-      <c r="L6" s="58"/>
+      <c r="B6" s="72"/>
+      <c r="C6" s="73"/>
+      <c r="D6" s="73"/>
+      <c r="E6" s="73"/>
+      <c r="F6" s="73"/>
+      <c r="G6" s="73"/>
+      <c r="H6" s="73"/>
+      <c r="I6" s="73"/>
+      <c r="J6" s="73"/>
+      <c r="K6" s="73"/>
+      <c r="L6" s="74"/>
       <c r="Q6" s="20" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2"/>
-      <c r="B7" s="59" t="s">
+      <c r="B7" s="63" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="15"/>
@@ -6024,13 +5828,13 @@
       <c r="J7" s="15"/>
       <c r="K7" s="15"/>
       <c r="L7" s="16"/>
-      <c r="Q7" s="62" t="s">
+      <c r="Q7" s="70" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
-      <c r="B8" s="60"/>
+      <c r="B8" s="53"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
@@ -6041,35 +5845,35 @@
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="10"/>
-      <c r="Q8" s="62"/>
+      <c r="Q8" s="70"/>
     </row>
     <row r="9" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2"/>
-      <c r="B9" s="60"/>
+      <c r="B9" s="53"/>
       <c r="C9" s="5"/>
       <c r="D9" s="6"/>
-      <c r="E9" s="63" t="s">
+      <c r="E9" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="64"/>
-      <c r="G9" s="65"/>
+      <c r="F9" s="56"/>
+      <c r="G9" s="57"/>
       <c r="H9" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I9" s="63" t="s">
+      <c r="I9" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="J9" s="64"/>
-      <c r="K9" s="65"/>
+      <c r="J9" s="56"/>
+      <c r="K9" s="57"/>
       <c r="L9" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="Q9" s="62"/>
+      <c r="Q9" s="70"/>
     </row>
     <row r="10" spans="1:17" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2"/>
-      <c r="B10" s="60"/>
-      <c r="C10" s="66"/>
+      <c r="B10" s="53"/>
+      <c r="C10" s="58"/>
       <c r="D10" s="2"/>
       <c r="E10" s="30"/>
       <c r="F10" s="30"/>
@@ -6079,12 +5883,12 @@
       <c r="J10" s="30"/>
       <c r="K10" s="30"/>
       <c r="L10" s="10"/>
-      <c r="Q10" s="62"/>
+      <c r="Q10" s="70"/>
     </row>
     <row r="11" spans="1:17" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2"/>
-      <c r="B11" s="60"/>
-      <c r="C11" s="67"/>
+      <c r="B11" s="53"/>
+      <c r="C11" s="59"/>
       <c r="D11" s="31" t="s">
         <v>11</v>
       </c>
@@ -6104,12 +5908,12 @@
       <c r="L11" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="Q11" s="62"/>
+      <c r="Q11" s="70"/>
     </row>
     <row r="12" spans="1:17" ht="5.0999999999999996" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
-      <c r="B12" s="61"/>
-      <c r="C12" s="68"/>
+      <c r="B12" s="54"/>
+      <c r="C12" s="61"/>
       <c r="D12" s="13"/>
       <c r="E12" s="18"/>
       <c r="F12" s="18"/>
@@ -6119,11 +5923,11 @@
       <c r="J12" s="18"/>
       <c r="K12" s="18"/>
       <c r="L12" s="14"/>
-      <c r="Q12" s="62"/>
+      <c r="Q12" s="70"/>
     </row>
     <row r="13" spans="1:17" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2"/>
-      <c r="B13" s="69" t="s">
+      <c r="B13" s="52" t="s">
         <v>15</v>
       </c>
       <c r="C13" s="2"/>
@@ -6136,11 +5940,11 @@
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="L13" s="10"/>
-      <c r="Q13" s="62"/>
+      <c r="Q13" s="70"/>
     </row>
     <row r="14" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2"/>
-      <c r="B14" s="60"/>
+      <c r="B14" s="53"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
@@ -6151,35 +5955,35 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
       <c r="L14" s="10"/>
-      <c r="Q14" s="62"/>
+      <c r="Q14" s="70"/>
     </row>
     <row r="15" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2"/>
-      <c r="B15" s="60"/>
+      <c r="B15" s="53"/>
       <c r="C15" s="5"/>
       <c r="D15" s="6"/>
-      <c r="E15" s="63" t="s">
+      <c r="E15" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="F15" s="64"/>
-      <c r="G15" s="65"/>
+      <c r="F15" s="56"/>
+      <c r="G15" s="57"/>
       <c r="H15" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I15" s="63" t="s">
+      <c r="I15" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="J15" s="64"/>
-      <c r="K15" s="65"/>
+      <c r="J15" s="56"/>
+      <c r="K15" s="57"/>
       <c r="L15" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="Q15" s="62"/>
+      <c r="Q15" s="70"/>
     </row>
     <row r="16" spans="1:17" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2"/>
-      <c r="B16" s="60"/>
-      <c r="C16" s="66"/>
+      <c r="B16" s="53"/>
+      <c r="C16" s="58"/>
       <c r="D16" s="2"/>
       <c r="E16" s="30"/>
       <c r="F16" s="30"/>
@@ -6189,12 +5993,12 @@
       <c r="J16" s="30"/>
       <c r="K16" s="30"/>
       <c r="L16" s="10"/>
-      <c r="Q16" s="62"/>
+      <c r="Q16" s="70"/>
     </row>
     <row r="17" spans="1:17" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2"/>
-      <c r="B17" s="60"/>
-      <c r="C17" s="67"/>
+      <c r="B17" s="53"/>
+      <c r="C17" s="59"/>
       <c r="D17" s="31" t="s">
         <v>11</v>
       </c>
@@ -6214,12 +6018,12 @@
       <c r="L17" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="Q17" s="62"/>
+      <c r="Q17" s="70"/>
     </row>
     <row r="18" spans="1:17" ht="5.0999999999999996" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
-      <c r="B18" s="61"/>
-      <c r="C18" s="68"/>
+      <c r="B18" s="54"/>
+      <c r="C18" s="61"/>
       <c r="D18" s="13"/>
       <c r="E18" s="18"/>
       <c r="F18" s="18"/>
@@ -6229,7 +6033,7 @@
       <c r="J18" s="18"/>
       <c r="K18" s="18"/>
       <c r="L18" s="14"/>
-      <c r="Q18" s="62"/>
+      <c r="Q18" s="70"/>
     </row>
     <row r="19" spans="1:17" ht="24.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2"/>
@@ -6244,7 +6048,7 @@
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
-      <c r="Q19" s="62"/>
+      <c r="Q19" s="70"/>
     </row>
     <row r="20" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>
@@ -6263,43 +6067,43 @@
     </row>
     <row r="21" spans="1:17" ht="28.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
-      <c r="B21" s="53" t="s">
+      <c r="B21" s="64" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="54"/>
-      <c r="D21" s="54"/>
-      <c r="E21" s="54"/>
-      <c r="F21" s="54"/>
-      <c r="G21" s="54"/>
-      <c r="H21" s="54"/>
-      <c r="I21" s="54"/>
-      <c r="J21" s="54"/>
-      <c r="K21" s="54"/>
-      <c r="L21" s="55"/>
+      <c r="C21" s="65"/>
+      <c r="D21" s="65"/>
+      <c r="E21" s="65"/>
+      <c r="F21" s="65"/>
+      <c r="G21" s="65"/>
+      <c r="H21" s="65"/>
+      <c r="I21" s="65"/>
+      <c r="J21" s="65"/>
+      <c r="K21" s="65"/>
+      <c r="L21" s="66"/>
       <c r="Q21" s="22" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:17" ht="28.35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
-      <c r="B22" s="70"/>
-      <c r="C22" s="71"/>
-      <c r="D22" s="71"/>
-      <c r="E22" s="71"/>
-      <c r="F22" s="71"/>
-      <c r="G22" s="71"/>
-      <c r="H22" s="71"/>
-      <c r="I22" s="71"/>
-      <c r="J22" s="71"/>
-      <c r="K22" s="71"/>
-      <c r="L22" s="72"/>
-      <c r="Q22" s="62" t="s">
+      <c r="B22" s="67"/>
+      <c r="C22" s="68"/>
+      <c r="D22" s="68"/>
+      <c r="E22" s="68"/>
+      <c r="F22" s="68"/>
+      <c r="G22" s="68"/>
+      <c r="H22" s="68"/>
+      <c r="I22" s="68"/>
+      <c r="J22" s="68"/>
+      <c r="K22" s="68"/>
+      <c r="L22" s="69"/>
+      <c r="Q22" s="70" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="23" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2"/>
-      <c r="B23" s="69" t="s">
+      <c r="B23" s="52" t="s">
         <v>15</v>
       </c>
       <c r="C23" s="2"/>
@@ -6312,35 +6116,35 @@
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
       <c r="L23" s="10"/>
-      <c r="Q23" s="62"/>
+      <c r="Q23" s="70"/>
     </row>
     <row r="24" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2"/>
-      <c r="B24" s="60"/>
+      <c r="B24" s="53"/>
       <c r="C24" s="5"/>
       <c r="D24" s="6"/>
-      <c r="E24" s="63" t="s">
+      <c r="E24" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="F24" s="64"/>
-      <c r="G24" s="65"/>
+      <c r="F24" s="56"/>
+      <c r="G24" s="57"/>
       <c r="H24" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I24" s="63" t="s">
+      <c r="I24" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="J24" s="64"/>
-      <c r="K24" s="65"/>
+      <c r="J24" s="56"/>
+      <c r="K24" s="57"/>
       <c r="L24" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="Q24" s="62"/>
+      <c r="Q24" s="70"/>
     </row>
     <row r="25" spans="1:17" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2"/>
-      <c r="B25" s="60"/>
-      <c r="C25" s="66"/>
+      <c r="B25" s="53"/>
+      <c r="C25" s="58"/>
       <c r="D25" s="2"/>
       <c r="E25" s="30"/>
       <c r="F25" s="30"/>
@@ -6350,12 +6154,12 @@
       <c r="J25" s="30"/>
       <c r="K25" s="30"/>
       <c r="L25" s="10"/>
-      <c r="Q25" s="62"/>
+      <c r="Q25" s="70"/>
     </row>
     <row r="26" spans="1:17" ht="15" x14ac:dyDescent="0.2">
       <c r="A26" s="2"/>
-      <c r="B26" s="60"/>
-      <c r="C26" s="67"/>
+      <c r="B26" s="53"/>
+      <c r="C26" s="59"/>
       <c r="D26" s="31" t="s">
         <v>19</v>
       </c>
@@ -6375,12 +6179,12 @@
       <c r="L26" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="Q26" s="62"/>
+      <c r="Q26" s="70"/>
     </row>
     <row r="27" spans="1:17" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2"/>
-      <c r="B27" s="60"/>
-      <c r="C27" s="73"/>
+      <c r="B27" s="53"/>
+      <c r="C27" s="60"/>
       <c r="D27" s="37"/>
       <c r="E27" s="7"/>
       <c r="F27" s="7"/>
@@ -6390,12 +6194,12 @@
       <c r="J27" s="7"/>
       <c r="K27" s="7"/>
       <c r="L27" s="38"/>
-      <c r="Q27" s="62"/>
+      <c r="Q27" s="70"/>
     </row>
     <row r="28" spans="1:17" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2"/>
-      <c r="B28" s="60"/>
-      <c r="C28" s="67"/>
+      <c r="B28" s="53"/>
+      <c r="C28" s="59"/>
       <c r="D28" s="2"/>
       <c r="E28" s="30"/>
       <c r="F28" s="30"/>
@@ -6405,12 +6209,12 @@
       <c r="J28" s="30"/>
       <c r="K28" s="30"/>
       <c r="L28" s="10"/>
-      <c r="Q28" s="62"/>
+      <c r="Q28" s="70"/>
     </row>
     <row r="29" spans="1:17" ht="15" x14ac:dyDescent="0.2">
       <c r="A29" s="2"/>
-      <c r="B29" s="60"/>
-      <c r="C29" s="67"/>
+      <c r="B29" s="53"/>
+      <c r="C29" s="59"/>
       <c r="D29" s="31" t="s">
         <v>20</v>
       </c>
@@ -6430,12 +6234,12 @@
       <c r="L29" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="Q29" s="62"/>
+      <c r="Q29" s="70"/>
     </row>
     <row r="30" spans="1:17" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
-      <c r="B30" s="60"/>
-      <c r="C30" s="73"/>
+      <c r="B30" s="53"/>
+      <c r="C30" s="60"/>
       <c r="D30" s="37"/>
       <c r="E30" s="7"/>
       <c r="F30" s="7"/>
@@ -6449,8 +6253,8 @@
     </row>
     <row r="31" spans="1:17" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2"/>
-      <c r="B31" s="60"/>
-      <c r="C31" s="67"/>
+      <c r="B31" s="53"/>
+      <c r="C31" s="59"/>
       <c r="D31" s="2"/>
       <c r="E31" s="30"/>
       <c r="F31" s="30"/>
@@ -6463,8 +6267,8 @@
     </row>
     <row r="32" spans="1:17" ht="15" x14ac:dyDescent="0.2">
       <c r="A32" s="2"/>
-      <c r="B32" s="60"/>
-      <c r="C32" s="67"/>
+      <c r="B32" s="53"/>
+      <c r="C32" s="59"/>
       <c r="D32" s="31" t="s">
         <v>22</v>
       </c>
@@ -6487,8 +6291,8 @@
     </row>
     <row r="33" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2"/>
-      <c r="B33" s="60"/>
-      <c r="C33" s="73"/>
+      <c r="B33" s="53"/>
+      <c r="C33" s="60"/>
       <c r="D33" s="37"/>
       <c r="E33" s="7"/>
       <c r="F33" s="7"/>
@@ -6501,8 +6305,8 @@
     </row>
     <row r="34" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2"/>
-      <c r="B34" s="60"/>
-      <c r="C34" s="67"/>
+      <c r="B34" s="53"/>
+      <c r="C34" s="59"/>
       <c r="D34" s="2"/>
       <c r="E34" s="30"/>
       <c r="F34" s="30"/>
@@ -6515,8 +6319,8 @@
     </row>
     <row r="35" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A35" s="2"/>
-      <c r="B35" s="60"/>
-      <c r="C35" s="67"/>
+      <c r="B35" s="53"/>
+      <c r="C35" s="59"/>
       <c r="D35" s="31" t="s">
         <v>23</v>
       </c>
@@ -6539,8 +6343,8 @@
     </row>
     <row r="36" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
-      <c r="B36" s="60"/>
-      <c r="C36" s="73"/>
+      <c r="B36" s="53"/>
+      <c r="C36" s="60"/>
       <c r="D36" s="37"/>
       <c r="E36" s="7"/>
       <c r="F36" s="7"/>
@@ -6553,8 +6357,8 @@
     </row>
     <row r="37" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2"/>
-      <c r="B37" s="60"/>
-      <c r="C37" s="67"/>
+      <c r="B37" s="53"/>
+      <c r="C37" s="59"/>
       <c r="D37" s="2"/>
       <c r="E37" s="30"/>
       <c r="F37" s="30"/>
@@ -6567,8 +6371,8 @@
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" s="2"/>
-      <c r="B38" s="60"/>
-      <c r="C38" s="67"/>
+      <c r="B38" s="53"/>
+      <c r="C38" s="59"/>
       <c r="D38" s="31" t="s">
         <v>25</v>
       </c>
@@ -6583,7 +6387,7 @@
     </row>
     <row r="39" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2"/>
-      <c r="B39" s="60"/>
+      <c r="B39" s="53"/>
       <c r="C39" s="35"/>
       <c r="D39" s="31"/>
       <c r="E39" s="30"/>
@@ -6597,7 +6401,7 @@
     </row>
     <row r="40" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A40" s="2"/>
-      <c r="B40" s="60"/>
+      <c r="B40" s="53"/>
       <c r="C40" s="35"/>
       <c r="D40" s="32" t="s">
         <v>26</v>
@@ -6621,7 +6425,7 @@
     </row>
     <row r="41" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2"/>
-      <c r="B41" s="60"/>
+      <c r="B41" s="53"/>
       <c r="C41" s="35"/>
       <c r="D41" s="27"/>
       <c r="E41" s="7"/>
@@ -6635,7 +6439,7 @@
     </row>
     <row r="42" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2"/>
-      <c r="B42" s="60"/>
+      <c r="B42" s="53"/>
       <c r="C42" s="35"/>
       <c r="D42" s="31"/>
       <c r="E42" s="30"/>
@@ -6649,7 +6453,7 @@
     </row>
     <row r="43" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A43" s="2"/>
-      <c r="B43" s="60"/>
+      <c r="B43" s="53"/>
       <c r="C43" s="35"/>
       <c r="D43" s="32" t="s">
         <v>28</v>
@@ -6673,7 +6477,7 @@
     </row>
     <row r="44" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2"/>
-      <c r="B44" s="60"/>
+      <c r="B44" s="53"/>
       <c r="C44" s="35"/>
       <c r="D44" s="27"/>
       <c r="E44" s="7"/>
@@ -6687,7 +6491,7 @@
     </row>
     <row r="45" spans="1:12" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2"/>
-      <c r="B45" s="60"/>
+      <c r="B45" s="53"/>
       <c r="C45" s="35"/>
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
@@ -6701,7 +6505,7 @@
     </row>
     <row r="46" spans="1:12" ht="5.0999999999999996" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2"/>
-      <c r="B46" s="61"/>
+      <c r="B46" s="54"/>
       <c r="C46" s="36"/>
       <c r="D46" s="13"/>
       <c r="E46" s="13"/>
@@ -6715,7 +6519,7 @@
     </row>
     <row r="47" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2"/>
-      <c r="B47" s="59" t="s">
+      <c r="B47" s="63" t="s">
         <v>6</v>
       </c>
       <c r="C47" s="15"/>
@@ -6731,30 +6535,30 @@
     </row>
     <row r="48" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2"/>
-      <c r="B48" s="60"/>
+      <c r="B48" s="53"/>
       <c r="C48" s="5"/>
       <c r="D48" s="6"/>
-      <c r="E48" s="63" t="s">
+      <c r="E48" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="F48" s="64"/>
-      <c r="G48" s="65"/>
+      <c r="F48" s="56"/>
+      <c r="G48" s="57"/>
       <c r="H48" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I48" s="63" t="s">
+      <c r="I48" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="J48" s="64"/>
-      <c r="K48" s="65"/>
+      <c r="J48" s="56"/>
+      <c r="K48" s="57"/>
       <c r="L48" s="11" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="49" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="2"/>
-      <c r="B49" s="60"/>
-      <c r="C49" s="66"/>
+      <c r="B49" s="53"/>
+      <c r="C49" s="58"/>
       <c r="D49" s="2"/>
       <c r="E49" s="30"/>
       <c r="F49" s="30"/>
@@ -6767,8 +6571,8 @@
     </row>
     <row r="50" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A50" s="2"/>
-      <c r="B50" s="60"/>
-      <c r="C50" s="67"/>
+      <c r="B50" s="53"/>
+      <c r="C50" s="59"/>
       <c r="D50" s="31" t="s">
         <v>19</v>
       </c>
@@ -6791,8 +6595,8 @@
     </row>
     <row r="51" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="2"/>
-      <c r="B51" s="60"/>
-      <c r="C51" s="73"/>
+      <c r="B51" s="53"/>
+      <c r="C51" s="60"/>
       <c r="D51" s="37"/>
       <c r="E51" s="7"/>
       <c r="F51" s="7"/>
@@ -6805,8 +6609,8 @@
     </row>
     <row r="52" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2"/>
-      <c r="B52" s="60"/>
-      <c r="C52" s="67"/>
+      <c r="B52" s="53"/>
+      <c r="C52" s="59"/>
       <c r="D52" s="2"/>
       <c r="E52" s="30"/>
       <c r="F52" s="30"/>
@@ -6819,8 +6623,8 @@
     </row>
     <row r="53" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A53" s="2"/>
-      <c r="B53" s="60"/>
-      <c r="C53" s="67"/>
+      <c r="B53" s="53"/>
+      <c r="C53" s="59"/>
       <c r="D53" s="31" t="s">
         <v>20</v>
       </c>
@@ -6843,8 +6647,8 @@
     </row>
     <row r="54" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="2"/>
-      <c r="B54" s="60"/>
-      <c r="C54" s="73"/>
+      <c r="B54" s="53"/>
+      <c r="C54" s="60"/>
       <c r="D54" s="37"/>
       <c r="E54" s="7"/>
       <c r="F54" s="7"/>
@@ -6857,8 +6661,8 @@
     </row>
     <row r="55" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="2"/>
-      <c r="B55" s="60"/>
-      <c r="C55" s="67"/>
+      <c r="B55" s="53"/>
+      <c r="C55" s="59"/>
       <c r="D55" s="2"/>
       <c r="E55" s="30"/>
       <c r="F55" s="30"/>
@@ -6871,8 +6675,8 @@
     </row>
     <row r="56" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A56" s="2"/>
-      <c r="B56" s="60"/>
-      <c r="C56" s="67"/>
+      <c r="B56" s="53"/>
+      <c r="C56" s="59"/>
       <c r="D56" s="31" t="s">
         <v>22</v>
       </c>
@@ -6895,8 +6699,8 @@
     </row>
     <row r="57" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="2"/>
-      <c r="B57" s="60"/>
-      <c r="C57" s="73"/>
+      <c r="B57" s="53"/>
+      <c r="C57" s="60"/>
       <c r="D57" s="37"/>
       <c r="E57" s="7"/>
       <c r="F57" s="7"/>
@@ -6909,8 +6713,8 @@
     </row>
     <row r="58" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="2"/>
-      <c r="B58" s="60"/>
-      <c r="C58" s="67"/>
+      <c r="B58" s="53"/>
+      <c r="C58" s="59"/>
       <c r="D58" s="2"/>
       <c r="E58" s="30"/>
       <c r="F58" s="30"/>
@@ -6923,8 +6727,8 @@
     </row>
     <row r="59" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A59" s="2"/>
-      <c r="B59" s="60"/>
-      <c r="C59" s="67"/>
+      <c r="B59" s="53"/>
+      <c r="C59" s="59"/>
       <c r="D59" s="31" t="s">
         <v>23</v>
       </c>
@@ -6947,8 +6751,8 @@
     </row>
     <row r="60" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="2"/>
-      <c r="B60" s="60"/>
-      <c r="C60" s="73"/>
+      <c r="B60" s="53"/>
+      <c r="C60" s="60"/>
       <c r="D60" s="37"/>
       <c r="E60" s="7"/>
       <c r="F60" s="7"/>
@@ -6961,8 +6765,8 @@
     </row>
     <row r="61" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="2"/>
-      <c r="B61" s="60"/>
-      <c r="C61" s="67"/>
+      <c r="B61" s="53"/>
+      <c r="C61" s="59"/>
       <c r="D61" s="2"/>
       <c r="E61" s="30"/>
       <c r="F61" s="30"/>
@@ -6975,8 +6779,8 @@
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A62" s="2"/>
-      <c r="B62" s="60"/>
-      <c r="C62" s="67"/>
+      <c r="B62" s="53"/>
+      <c r="C62" s="59"/>
       <c r="D62" s="31" t="s">
         <v>25</v>
       </c>
@@ -6991,7 +6795,7 @@
     </row>
     <row r="63" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="2"/>
-      <c r="B63" s="60"/>
+      <c r="B63" s="53"/>
       <c r="C63" s="35"/>
       <c r="D63" s="31"/>
       <c r="E63" s="30"/>
@@ -7005,7 +6809,7 @@
     </row>
     <row r="64" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A64" s="2"/>
-      <c r="B64" s="60"/>
+      <c r="B64" s="53"/>
       <c r="C64" s="35"/>
       <c r="D64" s="32" t="s">
         <v>26</v>
@@ -7029,7 +6833,7 @@
     </row>
     <row r="65" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="2"/>
-      <c r="B65" s="60"/>
+      <c r="B65" s="53"/>
       <c r="C65" s="35"/>
       <c r="D65" s="27"/>
       <c r="E65" s="7"/>
@@ -7043,7 +6847,7 @@
     </row>
     <row r="66" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="2"/>
-      <c r="B66" s="60"/>
+      <c r="B66" s="53"/>
       <c r="C66" s="35"/>
       <c r="D66" s="31"/>
       <c r="E66" s="30"/>
@@ -7057,7 +6861,7 @@
     </row>
     <row r="67" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A67" s="2"/>
-      <c r="B67" s="60"/>
+      <c r="B67" s="53"/>
       <c r="C67" s="35"/>
       <c r="D67" s="32" t="s">
         <v>30</v>
@@ -7081,7 +6885,7 @@
     </row>
     <row r="68" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="2"/>
-      <c r="B68" s="60"/>
+      <c r="B68" s="53"/>
       <c r="C68" s="35"/>
       <c r="D68" s="27"/>
       <c r="E68" s="7"/>
@@ -7095,7 +6899,7 @@
     </row>
     <row r="69" spans="1:12" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="2"/>
-      <c r="B69" s="60"/>
+      <c r="B69" s="53"/>
       <c r="C69" s="35"/>
       <c r="D69" s="2"/>
       <c r="E69" s="2"/>
@@ -7109,7 +6913,7 @@
     </row>
     <row r="70" spans="1:12" ht="5.0999999999999996" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2"/>
-      <c r="B70" s="61"/>
+      <c r="B70" s="54"/>
       <c r="C70" s="36"/>
       <c r="D70" s="13"/>
       <c r="E70" s="13"/>
@@ -7151,37 +6955,37 @@
     </row>
     <row r="73" spans="1:12" ht="28.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2"/>
-      <c r="B73" s="53" t="s">
+      <c r="B73" s="64" t="s">
         <v>32</v>
       </c>
-      <c r="C73" s="54"/>
-      <c r="D73" s="54"/>
-      <c r="E73" s="54"/>
-      <c r="F73" s="54"/>
-      <c r="G73" s="54"/>
-      <c r="H73" s="54"/>
-      <c r="I73" s="54"/>
-      <c r="J73" s="54"/>
-      <c r="K73" s="54"/>
-      <c r="L73" s="55"/>
+      <c r="C73" s="65"/>
+      <c r="D73" s="65"/>
+      <c r="E73" s="65"/>
+      <c r="F73" s="65"/>
+      <c r="G73" s="65"/>
+      <c r="H73" s="65"/>
+      <c r="I73" s="65"/>
+      <c r="J73" s="65"/>
+      <c r="K73" s="65"/>
+      <c r="L73" s="66"/>
     </row>
     <row r="74" spans="1:12" ht="28.35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="2"/>
-      <c r="B74" s="70"/>
-      <c r="C74" s="71"/>
-      <c r="D74" s="71"/>
-      <c r="E74" s="71"/>
-      <c r="F74" s="71"/>
-      <c r="G74" s="71"/>
-      <c r="H74" s="71"/>
-      <c r="I74" s="71"/>
-      <c r="J74" s="71"/>
-      <c r="K74" s="71"/>
-      <c r="L74" s="72"/>
+      <c r="B74" s="67"/>
+      <c r="C74" s="68"/>
+      <c r="D74" s="68"/>
+      <c r="E74" s="68"/>
+      <c r="F74" s="68"/>
+      <c r="G74" s="68"/>
+      <c r="H74" s="68"/>
+      <c r="I74" s="68"/>
+      <c r="J74" s="68"/>
+      <c r="K74" s="68"/>
+      <c r="L74" s="69"/>
     </row>
     <row r="75" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="2"/>
-      <c r="B75" s="69" t="s">
+      <c r="B75" s="52" t="s">
         <v>15</v>
       </c>
       <c r="C75" s="2"/>
@@ -7197,30 +7001,30 @@
     </row>
     <row r="76" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="2"/>
-      <c r="B76" s="60"/>
+      <c r="B76" s="53"/>
       <c r="C76" s="5"/>
       <c r="D76" s="6"/>
-      <c r="E76" s="63" t="s">
+      <c r="E76" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="F76" s="64"/>
-      <c r="G76" s="65"/>
+      <c r="F76" s="56"/>
+      <c r="G76" s="57"/>
       <c r="H76" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I76" s="63" t="s">
+      <c r="I76" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="J76" s="64"/>
-      <c r="K76" s="65"/>
+      <c r="J76" s="56"/>
+      <c r="K76" s="57"/>
       <c r="L76" s="11" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="77" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="2"/>
-      <c r="B77" s="60"/>
-      <c r="C77" s="66"/>
+      <c r="B77" s="53"/>
+      <c r="C77" s="58"/>
       <c r="D77" s="2"/>
       <c r="E77" s="30"/>
       <c r="F77" s="30"/>
@@ -7233,8 +7037,8 @@
     </row>
     <row r="78" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A78" s="2"/>
-      <c r="B78" s="60"/>
-      <c r="C78" s="67"/>
+      <c r="B78" s="53"/>
+      <c r="C78" s="59"/>
       <c r="D78" s="31" t="s">
         <v>33</v>
       </c>
@@ -7257,8 +7061,8 @@
     </row>
     <row r="79" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="2"/>
-      <c r="B79" s="60"/>
-      <c r="C79" s="73"/>
+      <c r="B79" s="53"/>
+      <c r="C79" s="60"/>
       <c r="D79" s="37"/>
       <c r="E79" s="7"/>
       <c r="F79" s="7"/>
@@ -7271,8 +7075,8 @@
     </row>
     <row r="80" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="2"/>
-      <c r="B80" s="60"/>
-      <c r="C80" s="67"/>
+      <c r="B80" s="53"/>
+      <c r="C80" s="59"/>
       <c r="D80" s="2"/>
       <c r="E80" s="30"/>
       <c r="F80" s="30"/>
@@ -7285,8 +7089,8 @@
     </row>
     <row r="81" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A81" s="2"/>
-      <c r="B81" s="60"/>
-      <c r="C81" s="67"/>
+      <c r="B81" s="53"/>
+      <c r="C81" s="59"/>
       <c r="D81" s="31" t="s">
         <v>34</v>
       </c>
@@ -7309,8 +7113,8 @@
     </row>
     <row r="82" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="2"/>
-      <c r="B82" s="74"/>
-      <c r="C82" s="73"/>
+      <c r="B82" s="62"/>
+      <c r="C82" s="60"/>
       <c r="D82" s="37"/>
       <c r="E82" s="7"/>
       <c r="F82" s="7"/>
@@ -7323,7 +7127,7 @@
     </row>
     <row r="83" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="2"/>
-      <c r="B83" s="69" t="s">
+      <c r="B83" s="52" t="s">
         <v>6</v>
       </c>
       <c r="C83" s="2"/>
@@ -7339,30 +7143,30 @@
     </row>
     <row r="84" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="2"/>
-      <c r="B84" s="60"/>
+      <c r="B84" s="53"/>
       <c r="C84" s="5"/>
       <c r="D84" s="6"/>
-      <c r="E84" s="63" t="s">
+      <c r="E84" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="F84" s="64"/>
-      <c r="G84" s="65"/>
+      <c r="F84" s="56"/>
+      <c r="G84" s="57"/>
       <c r="H84" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I84" s="63" t="s">
+      <c r="I84" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="J84" s="64"/>
-      <c r="K84" s="65"/>
+      <c r="J84" s="56"/>
+      <c r="K84" s="57"/>
       <c r="L84" s="11" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="85" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="2"/>
-      <c r="B85" s="60"/>
-      <c r="C85" s="66"/>
+      <c r="B85" s="53"/>
+      <c r="C85" s="58"/>
       <c r="D85" s="2"/>
       <c r="E85" s="30"/>
       <c r="F85" s="30"/>
@@ -7375,8 +7179,8 @@
     </row>
     <row r="86" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A86" s="2"/>
-      <c r="B86" s="60"/>
-      <c r="C86" s="67"/>
+      <c r="B86" s="53"/>
+      <c r="C86" s="59"/>
       <c r="D86" s="31" t="s">
         <v>33</v>
       </c>
@@ -7399,8 +7203,8 @@
     </row>
     <row r="87" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="2"/>
-      <c r="B87" s="60"/>
-      <c r="C87" s="73"/>
+      <c r="B87" s="53"/>
+      <c r="C87" s="60"/>
       <c r="D87" s="37"/>
       <c r="E87" s="7"/>
       <c r="F87" s="7"/>
@@ -7413,8 +7217,8 @@
     </row>
     <row r="88" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="2"/>
-      <c r="B88" s="60"/>
-      <c r="C88" s="67"/>
+      <c r="B88" s="53"/>
+      <c r="C88" s="59"/>
       <c r="D88" s="2"/>
       <c r="E88" s="30"/>
       <c r="F88" s="30"/>
@@ -7427,8 +7231,8 @@
     </row>
     <row r="89" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A89" s="2"/>
-      <c r="B89" s="60"/>
-      <c r="C89" s="67"/>
+      <c r="B89" s="53"/>
+      <c r="C89" s="59"/>
       <c r="D89" s="31" t="s">
         <v>34</v>
       </c>
@@ -7451,8 +7255,8 @@
     </row>
     <row r="90" spans="1:12" ht="5.0999999999999996" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2"/>
-      <c r="B90" s="61"/>
-      <c r="C90" s="68"/>
+      <c r="B90" s="54"/>
+      <c r="C90" s="61"/>
       <c r="D90" s="13"/>
       <c r="E90" s="18"/>
       <c r="F90" s="18"/>
@@ -8251,37 +8055,6 @@
   <sheetProtection algorithmName="SHA-512" hashValue="jUzRW1wZU4UKDlrc+ZcjfI1CGFMPpb3WBOiNrGujdLz4z6mGk5OrV9Q3LSR9/vcnYNn7Umyfq3hCTh4LwP0m/Q==" saltValue="0LYgXzE3BB0FL5cMFmUsdQ==" spinCount="100000" sheet="1" objects="1" scenarios="1" formatCells="0"/>
   <dataConsolidate/>
   <mergeCells count="43">
-    <mergeCell ref="B83:B90"/>
-    <mergeCell ref="E84:G84"/>
-    <mergeCell ref="I84:K84"/>
-    <mergeCell ref="C85:C87"/>
-    <mergeCell ref="C88:C90"/>
-    <mergeCell ref="B75:B82"/>
-    <mergeCell ref="E76:G76"/>
-    <mergeCell ref="I76:K76"/>
-    <mergeCell ref="C77:C79"/>
-    <mergeCell ref="C80:C82"/>
-    <mergeCell ref="B47:B70"/>
-    <mergeCell ref="E48:G48"/>
-    <mergeCell ref="C61:C62"/>
-    <mergeCell ref="B73:L73"/>
-    <mergeCell ref="B74:L74"/>
-    <mergeCell ref="I48:K48"/>
-    <mergeCell ref="C49:C51"/>
-    <mergeCell ref="C52:C54"/>
-    <mergeCell ref="C55:C57"/>
-    <mergeCell ref="C58:C60"/>
-    <mergeCell ref="B21:L21"/>
-    <mergeCell ref="B22:L22"/>
-    <mergeCell ref="Q22:Q29"/>
-    <mergeCell ref="B23:B46"/>
-    <mergeCell ref="E24:G24"/>
-    <mergeCell ref="I24:K24"/>
-    <mergeCell ref="C25:C27"/>
-    <mergeCell ref="C28:C30"/>
-    <mergeCell ref="C31:C33"/>
-    <mergeCell ref="C34:C36"/>
-    <mergeCell ref="C37:C38"/>
     <mergeCell ref="B1:L1"/>
     <mergeCell ref="B5:L5"/>
     <mergeCell ref="B6:L6"/>
@@ -8294,19 +8067,97 @@
     <mergeCell ref="E15:G15"/>
     <mergeCell ref="I15:K15"/>
     <mergeCell ref="C16:C18"/>
+    <mergeCell ref="B21:L21"/>
+    <mergeCell ref="B22:L22"/>
+    <mergeCell ref="Q22:Q29"/>
+    <mergeCell ref="B23:B46"/>
+    <mergeCell ref="E24:G24"/>
+    <mergeCell ref="I24:K24"/>
+    <mergeCell ref="C25:C27"/>
+    <mergeCell ref="C28:C30"/>
+    <mergeCell ref="C31:C33"/>
+    <mergeCell ref="C34:C36"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="B47:B70"/>
+    <mergeCell ref="E48:G48"/>
+    <mergeCell ref="C61:C62"/>
+    <mergeCell ref="B73:L73"/>
+    <mergeCell ref="B74:L74"/>
+    <mergeCell ref="I48:K48"/>
+    <mergeCell ref="C49:C51"/>
+    <mergeCell ref="C52:C54"/>
+    <mergeCell ref="C55:C57"/>
+    <mergeCell ref="C58:C60"/>
+    <mergeCell ref="B75:B82"/>
+    <mergeCell ref="E76:G76"/>
+    <mergeCell ref="I76:K76"/>
+    <mergeCell ref="C77:C79"/>
+    <mergeCell ref="C80:C82"/>
+    <mergeCell ref="B83:B90"/>
+    <mergeCell ref="E84:G84"/>
+    <mergeCell ref="I84:K84"/>
+    <mergeCell ref="C85:C87"/>
+    <mergeCell ref="C88:C90"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <customProperties>
-    <customPr name="IbpWorksheetKeyString_GUID" r:id="rId2"/>
-  </customProperties>
-  <drawing r:id="rId3"/>
-  <legacyDrawing r:id="rId4"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
   <controls>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27671" r:id="rId5" name="cbApplyOddEvenFormatting">
-          <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0" r:id="rId6">
+        <control shapeId="27649" r:id="rId4" name="cbApplyLevelFormatting">
+          <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0" r:id="rId5">
+            <anchor moveWithCells="1">
+              <from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>266700</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>66675</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>66675</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>342900</xdr:rowOff>
+              </to>
+            </anchor>
+          </controlPr>
+        </control>
+      </mc:Choice>
+      <mc:Fallback>
+        <control shapeId="27649" r:id="rId4" name="cbApplyLevelFormatting"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <control shapeId="27655" r:id="rId6" name="cbApplyMemberFormatting">
+          <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0" r:id="rId7">
+            <anchor moveWithCells="1">
+              <from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>266700</xdr:colOff>
+                <xdr:row>20</xdr:row>
+                <xdr:rowOff>66675</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>66675</xdr:colOff>
+                <xdr:row>20</xdr:row>
+                <xdr:rowOff>342900</xdr:rowOff>
+              </to>
+            </anchor>
+          </controlPr>
+        </control>
+      </mc:Choice>
+      <mc:Fallback>
+        <control shapeId="27655" r:id="rId6" name="cbApplyMemberFormatting"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <control shapeId="27671" r:id="rId8" name="cbApplyOddEvenFormatting">
+          <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0" r:id="rId9">
             <anchor moveWithCells="1">
               <from>
                 <xdr:col>1</xdr:col>
@@ -8325,62 +8176,12 @@
         </control>
       </mc:Choice>
       <mc:Fallback>
-        <control shapeId="27671" r:id="rId5" name="cbApplyOddEvenFormatting"/>
+        <control shapeId="27671" r:id="rId8" name="cbApplyOddEvenFormatting"/>
       </mc:Fallback>
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27655" r:id="rId7" name="cbApplyMemberFormatting">
-          <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0" r:id="rId8">
-            <anchor moveWithCells="1">
-              <from>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>266700</xdr:colOff>
-                <xdr:row>20</xdr:row>
-                <xdr:rowOff>66675</xdr:rowOff>
-              </from>
-              <to>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>66675</xdr:colOff>
-                <xdr:row>20</xdr:row>
-                <xdr:rowOff>342900</xdr:rowOff>
-              </to>
-            </anchor>
-          </controlPr>
-        </control>
-      </mc:Choice>
-      <mc:Fallback>
-        <control shapeId="27655" r:id="rId7" name="cbApplyMemberFormatting"/>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice Requires="x14">
-        <control shapeId="27649" r:id="rId9" name="cbApplyLevelFormatting">
-          <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0" r:id="rId10">
-            <anchor moveWithCells="1">
-              <from>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>266700</xdr:colOff>
-                <xdr:row>4</xdr:row>
-                <xdr:rowOff>66675</xdr:rowOff>
-              </from>
-              <to>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>66675</xdr:colOff>
-                <xdr:row>4</xdr:row>
-                <xdr:rowOff>342900</xdr:rowOff>
-              </to>
-            </anchor>
-          </controlPr>
-        </control>
-      </mc:Choice>
-      <mc:Fallback>
-        <control shapeId="27649" r:id="rId9" name="cbApplyLevelFormatting"/>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice Requires="x14">
-        <control shapeId="27650" r:id="rId11" name="Group Box 2">
+        <control shapeId="27650" r:id="rId10" name="Group Box 2">
           <controlPr defaultSize="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -8402,7 +8203,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27651" r:id="rId12" name="obLevelRowFirst">
+        <control shapeId="27651" r:id="rId11" name="obLevelRowFirst">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1">
               <from>
@@ -8424,7 +8225,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27652" r:id="rId13" name="obLevelColumnFirst">
+        <control shapeId="27652" r:id="rId12" name="obLevelColumnFirst">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1">
               <from>
@@ -8446,7 +8247,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27653" r:id="rId14" name="cbUseDefaultLevelFirst">
+        <control shapeId="27653" r:id="rId13" name="cbUseDefaultLevelFirst">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -8468,7 +8269,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27654" r:id="rId15" name="cbUseDefaultLevelSecond">
+        <control shapeId="27654" r:id="rId14" name="cbUseDefaultLevelSecond">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -8490,7 +8291,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27656" r:id="rId16" name="Group Box 8">
+        <control shapeId="27656" r:id="rId15" name="Group Box 8">
           <controlPr defaultSize="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -8512,7 +8313,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27657" r:id="rId17" name="obMemberRowFirst">
+        <control shapeId="27657" r:id="rId16" name="obMemberRowFirst">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1">
               <from>
@@ -8534,7 +8335,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27658" r:id="rId18" name="obMemberColumnFirst">
+        <control shapeId="27658" r:id="rId17" name="obMemberColumnFirst">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1">
               <from>
@@ -8556,7 +8357,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27659" r:id="rId19" name="cbApplyCalculatedMemberFirst">
+        <control shapeId="27659" r:id="rId18" name="cbApplyCalculatedMemberFirst">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -8578,7 +8379,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27660" r:id="rId20" name="cbApplyImputableMemberFirst">
+        <control shapeId="27660" r:id="rId19" name="cbApplyImputableMemberFirst">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -8600,7 +8401,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27661" r:id="rId21" name="cbApplyLocalMemberFirst">
+        <control shapeId="27661" r:id="rId20" name="cbApplyLocalMemberFirst">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -8622,7 +8423,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27662" r:id="rId22" name="cbApplyChangedMemberFirst">
+        <control shapeId="27662" r:id="rId21" name="cbApplyChangedMemberFirst">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -8644,7 +8445,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27663" r:id="rId23" name="cbApplySpecificMemberFirst">
+        <control shapeId="27663" r:id="rId22" name="cbApplySpecificMemberFirst">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -8666,7 +8467,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27664" r:id="rId24" name="AddMemberFirst">
+        <control shapeId="27664" r:id="rId23" name="AddMemberFirst">
           <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
@@ -8688,7 +8489,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27665" r:id="rId25" name="cbApplyCalculatedMemberSecond">
+        <control shapeId="27665" r:id="rId24" name="cbApplyCalculatedMemberSecond">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -8710,7 +8511,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27666" r:id="rId26" name="cbApplyImputableMemberSecond">
+        <control shapeId="27666" r:id="rId25" name="cbApplyImputableMemberSecond">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -8732,7 +8533,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27667" r:id="rId27" name="cbApplyLocalMemberSecond">
+        <control shapeId="27667" r:id="rId26" name="cbApplyLocalMemberSecond">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -8754,7 +8555,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27668" r:id="rId28" name="cbApplyChangedMemberSecond">
+        <control shapeId="27668" r:id="rId27" name="cbApplyChangedMemberSecond">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -8776,7 +8577,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27669" r:id="rId29" name="cbApplySpecificMemberSecond">
+        <control shapeId="27669" r:id="rId28" name="cbApplySpecificMemberSecond">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -8798,7 +8599,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27670" r:id="rId30" name="AddMemberSecond">
+        <control shapeId="27670" r:id="rId29" name="AddMemberSecond">
           <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
@@ -8820,7 +8621,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27672" r:id="rId31" name="Group Box 24">
+        <control shapeId="27672" r:id="rId30" name="Group Box 24">
           <controlPr defaultSize="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -8842,7 +8643,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27673" r:id="rId32" name="obOddEvenRowFirst">
+        <control shapeId="27673" r:id="rId31" name="obOddEvenRowFirst">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1">
               <from>
@@ -8864,7 +8665,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27674" r:id="rId33" name="obOddEvenColumnFirst">
+        <control shapeId="27674" r:id="rId32" name="obOddEvenColumnFirst">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1">
               <from>
@@ -8886,7 +8687,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27675" r:id="rId34" name="cbUseOddFirst">
+        <control shapeId="27675" r:id="rId33" name="cbUseOddFirst">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -8908,7 +8709,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27676" r:id="rId35" name="cbUseEvenFirst">
+        <control shapeId="27676" r:id="rId34" name="cbUseEvenFirst">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -8930,7 +8731,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27677" r:id="rId36" name="cbUseOddSecond">
+        <control shapeId="27677" r:id="rId35" name="cbUseOddSecond">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -8952,7 +8753,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27678" r:id="rId37" name="cbUseEvenSecond">
+        <control shapeId="27678" r:id="rId36" name="cbUseEvenSecond">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -8974,7 +8775,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27679" r:id="rId38" name="AddedMember1_1">
+        <control shapeId="27679" r:id="rId37" name="AddedMember1_1">
           <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
@@ -8996,7 +8797,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27680" r:id="rId39" name="ChangeMember1_1">
+        <control shapeId="27680" r:id="rId38" name="ChangeMember1_1">
           <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
@@ -9018,7 +8819,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27681" r:id="rId40" name="UpMember1_1">
+        <control shapeId="27681" r:id="rId39" name="UpMember1_1">
           <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
@@ -9040,7 +8841,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27682" r:id="rId41" name="DownMember1_1">
+        <control shapeId="27682" r:id="rId40" name="DownMember1_1">
           <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
@@ -9062,7 +8863,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27683" r:id="rId42" name="AddedMember1_2">
+        <control shapeId="27683" r:id="rId41" name="AddedMember1_2">
           <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
@@ -9084,7 +8885,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27684" r:id="rId43" name="ChangeMember1_2">
+        <control shapeId="27684" r:id="rId42" name="ChangeMember1_2">
           <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
@@ -9106,7 +8907,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27685" r:id="rId44" name="UpMember1_2">
+        <control shapeId="27685" r:id="rId43" name="UpMember1_2">
           <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
@@ -9128,7 +8929,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27686" r:id="rId45" name="DownMember1_2">
+        <control shapeId="27686" r:id="rId44" name="DownMember1_2">
           <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
@@ -9150,7 +8951,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27687" r:id="rId46" name="AddedMember2_1">
+        <control shapeId="27687" r:id="rId45" name="AddedMember2_1">
           <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
@@ -9172,7 +8973,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27688" r:id="rId47" name="ChangeMember2_1">
+        <control shapeId="27688" r:id="rId46" name="ChangeMember2_1">
           <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
@@ -9194,7 +8995,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27689" r:id="rId48" name="UpMember2_1">
+        <control shapeId="27689" r:id="rId47" name="UpMember2_1">
           <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
@@ -9216,7 +9017,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27690" r:id="rId49" name="DownMember2_1">
+        <control shapeId="27690" r:id="rId48" name="DownMember2_1">
           <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
@@ -9238,7 +9039,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27691" r:id="rId50" name="AddedMember2_2">
+        <control shapeId="27691" r:id="rId49" name="AddedMember2_2">
           <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
@@ -9260,7 +9061,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27692" r:id="rId51" name="ChangeMember2_2">
+        <control shapeId="27692" r:id="rId50" name="ChangeMember2_2">
           <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
@@ -9282,7 +9083,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27693" r:id="rId52" name="UpMember2_2">
+        <control shapeId="27693" r:id="rId51" name="UpMember2_2">
           <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
@@ -9304,7 +9105,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27694" r:id="rId53" name="DownMember2_2">
+        <control shapeId="27694" r:id="rId52" name="DownMember2_2">
           <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="_xll.IBPXLClient.TechnicalCategory.ButtonActionInIBPClientFormattingSheet">
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
@@ -9326,7 +9127,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27695" r:id="rId54" name="cbApplyLevelFormattingShape">
+        <control shapeId="27695" r:id="rId53" name="cbApplyLevelFormattingShape">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -9348,7 +9149,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27696" r:id="rId55" name="cbApplyMemberFormattingShape">
+        <control shapeId="27696" r:id="rId54" name="cbApplyMemberFormattingShape">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -9370,7 +9171,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="27697" r:id="rId56" name="cbApplyOddEvenFormattingShape">
+        <control shapeId="27697" r:id="rId55" name="cbApplyOddEvenFormattingShape">
           <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
             <anchor moveWithCells="1">
               <from>
@@ -9395,7 +9196,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -9528,43 +9329,14 @@
   <pageSetup orientation="portrait" horizontalDpi="300" r:id="rId1"/>
   <customProperties>
     <customPr name="EpmWorksheetKeyString_GUID" r:id="rId2"/>
-    <customPr name="IbpWorksheetKeyString_GUID" r:id="rId3"/>
   </customProperties>
-  <drawing r:id="rId4"/>
-  <legacyDrawing r:id="rId5"/>
-  <picture r:id="rId6"/>
-  <controls>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice Requires="x14">
-        <control shapeId="3093" r:id="rId7" name="FPMExcelClientSheetOptionstb1">
-          <controlPr defaultSize="0" autoLine="0" r:id="rId8">
-            <anchor moveWithCells="1" sizeWithCells="1">
-              <from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>0</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>0</xdr:rowOff>
-              </from>
-              <to>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>0</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>0</xdr:rowOff>
-              </to>
-            </anchor>
-          </controlPr>
-        </control>
-      </mc:Choice>
-      <mc:Fallback>
-        <control shapeId="3093" r:id="rId7" name="FPMExcelClientSheetOptionstb1"/>
-      </mc:Fallback>
-    </mc:AlternateContent>
-  </controls>
+  <drawing r:id="rId3"/>
+  <picture r:id="rId4"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -9699,60 +9471,7 @@
     <customPr name="EpmWorksheetKeyString_GUID" r:id="rId2"/>
   </customProperties>
   <drawing r:id="rId3"/>
-  <legacyDrawing r:id="rId4"/>
-  <picture r:id="rId5"/>
-  <controls>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice Requires="x14">
-        <control shapeId="5127" r:id="rId6" name="TextBox2">
-          <controlPr defaultSize="0" disabled="1" autoLine="0" r:id="rId7">
-            <anchor>
-              <from>
-                <xdr:col>8</xdr:col>
-                <xdr:colOff>76200</xdr:colOff>
-                <xdr:row>5</xdr:row>
-                <xdr:rowOff>0</xdr:rowOff>
-              </from>
-              <to>
-                <xdr:col>8</xdr:col>
-                <xdr:colOff>85725</xdr:colOff>
-                <xdr:row>5</xdr:row>
-                <xdr:rowOff>9525</xdr:rowOff>
-              </to>
-            </anchor>
-          </controlPr>
-        </control>
-      </mc:Choice>
-      <mc:Fallback>
-        <control shapeId="5127" r:id="rId6" name="TextBox2"/>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice Requires="x14">
-        <control shapeId="5121" r:id="rId8" name="FPMExcelClientSheetOptionstb1">
-          <controlPr defaultSize="0" autoLine="0" r:id="rId9">
-            <anchor moveWithCells="1" sizeWithCells="1">
-              <from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>0</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>0</xdr:rowOff>
-              </from>
-              <to>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>0</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>0</xdr:rowOff>
-              </to>
-            </anchor>
-          </controlPr>
-        </control>
-      </mc:Choice>
-      <mc:Fallback>
-        <control shapeId="5121" r:id="rId8" name="FPMExcelClientSheetOptionstb1"/>
-      </mc:Fallback>
-    </mc:AlternateContent>
-  </controls>
+  <picture r:id="rId4"/>
 </worksheet>
 </file>
 

</xml_diff>